<commit_message>
test: add functional CLI test suite with fixtures and README docs
- Add src/tests/test_cli.py with 30 tests covering:
  init-db, generate-players, register-players, register-standings,
  generate-swiss-pairings, populate-results, and print-table commands
- Add src/tests/conftest.py with session-scoped fixtures:
  fresh_database (init on setup, DROP CASCADE on teardown),
  session_setup (players CSV + DB registration), num_players,
  set_working_directory, count_rows, scalar, read_csv
- Fix class-scoped fixture deprecation (PytestRemovedIn10Warning):
  convert run() to @classmethod using cls instead of self
- Ensure all class fixtures explicitly depend on session_setup
  to guarantee correct execution order across test classes
- Add Testing section to README covering prerequisites, env vars,
  how to run, fixture lifecycle, test class breakdown, CI setup,
  and troubleshooting guide
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -454,20 +454,20 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Aaron Duncan</t>
+          <t>Beth Castillo</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>13.5</v>
+        <v>19</v>
       </c>
       <c r="F2" t="n">
-        <v>4.5</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="3">
@@ -476,20 +476,20 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Stephen Bernard</t>
+          <t>Mr. Jonathan Gilbert</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D3" t="n">
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="F3" t="n">
-        <v>3.5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -498,20 +498,20 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Jessica Vega</t>
+          <t>John Gonzalez</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>13.5</v>
+        <v>19</v>
       </c>
       <c r="F4" t="n">
-        <v>3</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="5">
@@ -520,20 +520,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Brad Smith</t>
+          <t>Stephanie Burnett</t>
         </is>
       </c>
       <c r="C5" t="n">
+        <v>9</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>26</v>
+      </c>
+      <c r="F5" t="n">
         <v>5</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" t="n">
-        <v>11</v>
-      </c>
-      <c r="F5" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -542,20 +542,20 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Denise English</t>
+          <t>Steven Williams</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F6" t="n">
-        <v>2.5</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="7">
@@ -564,20 +564,20 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Amy Friedman</t>
+          <t>Trevor Robinson</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="F7" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="8">
@@ -586,20 +586,20 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Debra Jensen DDS</t>
+          <t>Alicia Turner</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D8" t="n">
         <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="F8" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -608,20 +608,20 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Timothy Levine</t>
+          <t>Christopher Pennington</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D9" t="n">
         <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>11.5</v>
+        <v>26</v>
       </c>
       <c r="F9" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="10">
@@ -630,20 +630,20 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>James Thompson</t>
+          <t>Rachel Goodwin</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D10" t="n">
         <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F10" t="n">
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="11">
@@ -652,20 +652,20 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Nicholas Cantu</t>
+          <t>Katie Goodwin</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D11" t="n">
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="F11" t="n">
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>